<commit_message>
Add Hammer and Poz content
</commit_message>
<xml_diff>
--- a/NULL_game_db.xlsx
+++ b/NULL_game_db.xlsx
@@ -19,17 +19,22 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="recipes" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="recipe_materials" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="system_rules" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEMPLATE_CHARACTER" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEMPLATE_SKILL" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEMPLATE_STAGE" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEMPLATE_DROP" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEMPLATE_RECIPE" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$B$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'characters'!$A$1:$H$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'character_levels'!$A$1:$E$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'traits'!$A$1:$C$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'skills'!$A$1:$G$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'skill_levels'!$A$1:$I$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'stages'!$A$1:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'stage_waves'!$A$1:$E$44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'drops'!$A$1:$E$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'characters'!$A$1:$H$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'character_levels'!$A$1:$E$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'traits'!$A$1:$C$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'skills'!$A$1:$G$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'skill_levels'!$A$1:$I$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'stages'!$A$1:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'stage_waves'!$A$1:$E$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'drops'!$A$1:$E$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'recipes'!$A$1:$D$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'recipe_materials'!$A$1:$C$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'system_rules'!$A$1:$C$6</definedName>
@@ -41,7 +46,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,8 +58,17 @@
       <b val="1"/>
       <color rgb="00E0FF00"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00E0FF00"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -66,8 +80,28 @@
         <fgColor rgb="00151515"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00080808"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00252525"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -75,15 +109,46 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00777777"/>
+      </left>
+      <right style="thin">
+        <color rgb="00777777"/>
+      </right>
+      <top style="thin">
+        <color rgb="00777777"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00777777"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -209,8 +274,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T_characters" displayName="T_characters" ref="A1:H7" headerRowCount="1">
-  <autoFilter ref="A1:H7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T_characters" displayName="T_characters" ref="A1:H9" headerRowCount="1">
+  <autoFilter ref="A1:H9"/>
   <tableColumns count="8">
     <tableColumn id="1" name="monster_id"/>
     <tableColumn id="2" name="name"/>
@@ -226,8 +291,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T_characterlevels" displayName="T_characterlevels" ref="A1:E13" headerRowCount="1">
-  <autoFilter ref="A1:E13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T_characterlevels" displayName="T_characterlevels" ref="A1:E17" headerRowCount="1">
+  <autoFilter ref="A1:E17"/>
   <tableColumns count="5">
     <tableColumn id="1" name="monster_id"/>
     <tableColumn id="2" name="level"/>
@@ -240,8 +305,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T_traits" displayName="T_traits" ref="A1:C8" headerRowCount="1">
-  <autoFilter ref="A1:C8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T_traits" displayName="T_traits" ref="A1:C10" headerRowCount="1">
+  <autoFilter ref="A1:C10"/>
   <tableColumns count="3">
     <tableColumn id="1" name="trait_id"/>
     <tableColumn id="2" name="name"/>
@@ -252,8 +317,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="T_skills" displayName="T_skills" ref="A1:G8" headerRowCount="1">
-  <autoFilter ref="A1:G8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="T_skills" displayName="T_skills" ref="A1:G10" headerRowCount="1">
+  <autoFilter ref="A1:G10"/>
   <tableColumns count="7">
     <tableColumn id="1" name="skill_id"/>
     <tableColumn id="2" name="name"/>
@@ -268,8 +333,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="T_skilllevels" displayName="T_skilllevels" ref="A1:I22" headerRowCount="1">
-  <autoFilter ref="A1:I22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="T_skilllevels" displayName="T_skilllevels" ref="A1:I28" headerRowCount="1">
+  <autoFilter ref="A1:I28"/>
   <tableColumns count="9">
     <tableColumn id="1" name="skill_id"/>
     <tableColumn id="2" name="level"/>
@@ -286,8 +351,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="T_stages" displayName="T_stages" ref="A1:F9" headerRowCount="1">
-  <autoFilter ref="A1:F9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="T_stages" displayName="T_stages" ref="A1:F13" headerRowCount="1">
+  <autoFilter ref="A1:F13"/>
   <tableColumns count="6">
     <tableColumn id="1" name="stage_id"/>
     <tableColumn id="2" name="name"/>
@@ -301,8 +366,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_stagewaves" displayName="T_stagewaves" ref="A1:E44" headerRowCount="1">
-  <autoFilter ref="A1:E44"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_stagewaves" displayName="T_stagewaves" ref="A1:E57" headerRowCount="1">
+  <autoFilter ref="A1:E57"/>
   <tableColumns count="5">
     <tableColumn id="1" name="stage_id"/>
     <tableColumn id="2" name="wave"/>
@@ -315,11 +380,11 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="T_drops" displayName="T_drops" ref="A1:E16" headerRowCount="1">
-  <autoFilter ref="A1:E16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="T_drops" displayName="T_drops" ref="A1:E33" headerRowCount="1">
+  <autoFilter ref="A1:E33"/>
   <tableColumns count="5">
     <tableColumn id="1" name="source_monster_id"/>
-    <tableColumn id="2" name="min_level"/>
+    <tableColumn id="2" name="source_level"/>
     <tableColumn id="3" name="drop_type"/>
     <tableColumn id="4" name="drop_id"/>
     <tableColumn id="5" name="rate"/>
@@ -1025,13 +1090,1455 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00E0FF00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>NEW CHARACTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>黄色セルを埋めます。確定後、characters / character_levels / traits へ転記してください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>入力</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>入力例</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>monster_id</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>M_NEWNAME</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>M_ + 英大文字。既存IDと重複不可</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>表示名</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>NewCharacter</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>ゲーム中に表示する名称</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>glyph</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>一覧や簡易描画で使う記号</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>基礎HP Lv1</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr"/>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Lv1のHP</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>基礎S Lv1</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr"/>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Lv1のスピード</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>スキル枠</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr"/>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>装備可能なスキル数</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Lv1特性ID</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr"/>
+      <c r="C11" s="6" t="inlineStr"/>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>通常は空欄。trait_idを指定可能</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr"/>
+      <c r="C12" s="6" t="inlineStr"/>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>キャラクター詳細文</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Lv2 HP加算</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr"/>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Lv1からの加算値</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Lv2 S加算</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr"/>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Lv1からの加算値</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Lv2 獲得特性ID</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr"/>
+      <c r="C15" s="6" t="inlineStr"/>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>新特性ならtraitsにも追加</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Lv3 HP加算</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr"/>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Lv2からの加算値</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Lv3 S加算</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr"/>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Lv2からの加算値</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Lv3 獲得特性ID</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr"/>
+      <c r="C18" s="6" t="inlineStr"/>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>新特性ならtraitsにも追加</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>特性名</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr"/>
+      <c r="C19" s="6" t="inlineStr"/>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>新特性を追加する場合</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>特性説明</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr"/>
+      <c r="C20" s="6" t="inlineStr"/>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>発動条件・効果・重複可否</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>見た目</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr"/>
+      <c r="C21" s="6" t="inlineStr"/>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>形状、線、ストライプ、色など</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>専用アニメーション</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr"/>
+      <c r="C22" s="6" t="inlineStr"/>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>攻撃・登場・被弾演出</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="入力値エラー" error="一覧から選択してください" type="list">
+      <formula1>"1,2,3"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00E0FF00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>NEW SKILL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>黄色セルを埋めます。確定後、skills / skill_levels へ転記してください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>入力</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>入力例</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>skill_id</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>SK_NEWNAME</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>SK_ + 英大文字。既存IDと重複不可</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>表示名</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>NewSkill</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>ゲーム中に表示する名称</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>glyph</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>◇</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>ボタンや一覧で使う記号</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr"/>
+      <c r="C8" s="6" t="inlineStr"/>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>プレイヤー向け効果文</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>対象</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr"/>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>enemy / ally / self</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>対象数</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr"/>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>同時に選ぶ対象数</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>効果タイプ</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr"/>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>damage / guard / hide / rapid / speed_buff / speed_strike / hp_strike / poison_attack</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Lv1 Power</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr"/>
+      <c r="C12" s="6" t="inlineStr"/>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>固定ダメージ系のみ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Lv1 CT</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr"/>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>使用後のクールタイム</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Lv1 倍率</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr"/>
+      <c r="C14" s="6" t="inlineStr"/>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>S倍率・連射倍率など。50%は0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Lv1 Hits</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr"/>
+      <c r="C15" s="6" t="inlineStr"/>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>連射回数</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Lv1 Guard%</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr"/>
+      <c r="C16" s="6" t="inlineStr"/>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>20%は0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Lv1 Speed%</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr"/>
+      <c r="C17" s="6" t="inlineStr"/>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>20%は0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Lv1 持続ターン</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr"/>
+      <c r="C18" s="6" t="inlineStr"/>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>バフなどの持続</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Lv2変更点</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr"/>
+      <c r="C19" s="6" t="inlineStr"/>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>CT、威力、倍率など</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Lv3変更点</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr"/>
+      <c r="C20" s="6" t="inlineStr"/>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>CT、威力、倍率など</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>専用アニメーション</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr"/>
+      <c r="C21" s="6" t="inlineStr"/>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>発動演出の指示</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="入力値エラー" error="一覧から選択してください" type="list">
+      <formula1>"enemy,ally,self"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="入力値エラー" error="一覧から選択してください" type="list">
+      <formula1>"damage,guard,hide,rapid,speed_buff,speed_strike,hp_strike,poison_attack"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00E0FF00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>NEW STAGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>上部にステージ情報、下部に敵を出現順で入力します。空行は無視してください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>入力</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>入力例</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>stage_id</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>STAGE_008</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>通常はSTAGE_、テーマはSP_</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>表示名</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>new stage</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>ステージ選択画面の名称</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>カテゴリ</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>normal / special</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr"/>
+      <c r="C8" s="6" t="inlineStr"/>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>ステージカードの概要</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>解放条件タイプ</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr"/>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>clear</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>always / clear / kills</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>解放条件値</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr"/>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>STAGE_007</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>clearならstage_id、killsなら M_ID:30;M_ID:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>wave</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>monster_id</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>level</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n"/>
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n"/>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n"/>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n"/>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="8" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="8" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n"/>
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="8" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n"/>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="8" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="n"/>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="8" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="8" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="8" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="8" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="n"/>
+      <c r="B29" s="8" t="n"/>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="8" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="n"/>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="8" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n"/>
+      <c r="B31" s="8" t="n"/>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="8" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n"/>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="8" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="n"/>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="8" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n"/>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="8" t="n"/>
+      <c r="D34" s="8" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="n"/>
+      <c r="B35" s="8" t="n"/>
+      <c r="C35" s="8" t="n"/>
+      <c r="D35" s="8" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n"/>
+      <c r="B36" s="8" t="n"/>
+      <c r="C36" s="8" t="n"/>
+      <c r="D36" s="8" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="n"/>
+      <c r="B37" s="8" t="n"/>
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="8" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="入力値エラー" error="一覧から選択してください" type="list">
+      <formula1>"normal,special"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="入力値エラー" error="一覧から選択してください" type="list">
+      <formula1>"always,clear,kills"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D14:D37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="入力値エラー" error="一覧から選択してください" type="list">
+      <formula1>"1,2,3"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00E0FF00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>NEW DROPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>敵Lvごとのドロップ候補を入力します。確率20%は0.2で入力してください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>source_monster_id</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>source_level</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>drop_type</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>drop_id</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="n"/>
+      <c r="B5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="n"/>
+      <c r="B6" s="8" t="n"/>
+      <c r="C6" s="8" t="n"/>
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="8" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="n"/>
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="n"/>
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="8" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n"/>
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="8" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n"/>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n"/>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="8" t="n"/>
+      <c r="E18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n"/>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="8" t="n"/>
+      <c r="E21" s="8" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="8" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n"/>
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="8" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n"/>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="8" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="B5:B24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="入力値エラー" error="一覧から選択してください" type="list">
+      <formula1>"1,2,3"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C5:C24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="入力値エラー" error="一覧から選択してください" type="list">
+      <formula1>"monster,skill,recipe"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00E0FF00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>NEW RECIPE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>レシピ本体と必要素材を入力します。素材は最大10種類まで記入できます。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>入力</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>入力例</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>説明</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>recipe_id</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>R_M_NEWNAME</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>R_M_キャラ / R_SK_スキル</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>表示名</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>NewRecipe</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>レシピ一覧の名称</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>結果タイプ</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>monster</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>monster / skill</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>結果ID</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr"/>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>M_NEWNAME</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>獲得するキャラまたはスキルID</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>material_monster_id</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="8" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n"/>
+      <c r="B15" s="8" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n"/>
+      <c r="B16" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n"/>
+      <c r="B17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n"/>
+      <c r="B18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n"/>
+      <c r="B20" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n"/>
+      <c r="B21" s="8" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="入力値エラー" error="一覧から選択してください" type="list">
+      <formula1>"monster,skill"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1040,7 +2547,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
     <col width="27" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -1278,8 +2785,76 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>M_HAMMER</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ハンマー</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1ターン溜めて強打を行う低速個体。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ポズ</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>♟</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>poisonSecretion</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>通常攻撃で毒を分泌する状態異常型個体。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H7"/>
+  <autoFilter ref="A1:H9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1293,14 +2868,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1562,8 +3137,80 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>M_HAMMER</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>M_HAMMER</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>heavyStrike</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" t="n">
+        <v>6</v>
+      </c>
+      <c r="D16" t="n">
+        <v>15</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" t="n">
+        <v>7</v>
+      </c>
+      <c r="D17" t="n">
+        <v>15</v>
+      </c>
+      <c r="E17" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E13"/>
+  <autoFilter ref="A1:E17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1577,12 +3224,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1721,8 +3368,42 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>heavyStrike</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>強打</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>通常攻撃を選ぶと1ターン溜め、次ターンに現在HPと同じダメージを与える。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>poisonSecretion</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>毒分泌</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>通常攻撃命中時、30%で対象を2ターン毒状態にする。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C8"/>
+  <autoFilter ref="A1:C10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1736,16 +3417,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2030,8 +3711,78 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SK_HEAVY_STRIKE</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>強打</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>1ターン溜め、次ターンに現在HPと同じダメージ。</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>hp_strike</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SK_POISON_SECRETION</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>分泌毒</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>♟</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>通常攻撃後、対象へ毒を確定付与。</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>enemy</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>poison_attack</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G8"/>
+  <autoFilter ref="A1:G10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2045,10 +3796,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -2553,8 +4304,158 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SK_HEAVY_STRIKE</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="n">
+        <v>8</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SK_HEAVY_STRIKE</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="n">
+        <v>7</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SK_HEAVY_STRIKE</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="n">
+        <v>6</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SK_POISON_SECRETION</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="n">
+        <v>5</v>
+      </c>
+      <c r="D26" t="n">
+        <v>6</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SK_POISON_SECRETION</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" t="n">
+        <v>5</v>
+      </c>
+      <c r="D27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SK_POISON_SECRETION</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" t="n">
+        <v>5</v>
+      </c>
+      <c r="D28" t="n">
+        <v>4</v>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I22"/>
+  <autoFilter ref="A1:I28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2568,7 +4469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2863,8 +4764,128 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>STAGE_008</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>鍛冶</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1 WAVE / ハンマー Lv1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>STAGE_009</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>工房</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2 WAVES / ハンマー Lv2-3</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>clear</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>STAGE_008</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>STAGE_010</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>工業廃水</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1 WAVE / ポズ Lv1</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>STAGE_011</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>毒沼</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>3 WAVES / ポズ Lv2-3</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>clear</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>STAGE_010</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F9"/>
+  <autoFilter ref="A1:F13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2878,7 +4899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3818,8 +5839,281 @@
         <v>3</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>STAGE_008</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>M_HAMMER</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>STAGE_009</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>M_HAMMER</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>STAGE_009</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>M_HAMMER</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>STAGE_009</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>M_HAMMER</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>STAGE_009</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" t="n">
+        <v>2</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>M_HAMMER</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>STAGE_009</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>M_HAMMER</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>STAGE_010</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>STAGE_011</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>STAGE_011</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" t="n">
+        <v>2</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>STAGE_011</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>STAGE_011</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>3</v>
+      </c>
+      <c r="C55" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>STAGE_011</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>STAGE_011</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>3</v>
+      </c>
+      <c r="C57" t="n">
+        <v>3</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E44"/>
+  <autoFilter ref="A1:E57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3833,13 +6127,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -3851,7 +6145,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>min_level</t>
+          <t>source_level</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -3896,11 +6190,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>M_BLACKSQUARE</t>
+          <t>M_BLACKCIRCLE</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3909,7 +6203,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>M_BLACKSQUARE</t>
+          <t>M_BLACKCIRCLE</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -3919,7 +6213,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>M_BLACKSQUARE</t>
+          <t>M_BLACKCIRCLE</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -3927,22 +6221,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>monster</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SK_BLACKSQUARE</t>
+          <t>M_BLACKCIRCLE</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>M_HIDER</t>
+          <t>M_BLACKSQUARE</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -3955,7 +6249,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>M_HIDER</t>
+          <t>M_BLACKSQUARE</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -3965,34 +6259,34 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>M_HIDER</t>
+          <t>M_BLACKSQUARE</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>monster</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SK_HIDE</t>
+          <t>M_BLACKSQUARE</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>M_BLACKTRIANGLE</t>
+          <t>M_BLACKSQUARE</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -4001,7 +6295,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>M_BLACKTRIANGLE</t>
+          <t>M_BLACKSQUARE</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -4011,7 +6305,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>M_BLACKTRIANGLE</t>
+          <t>M_BLACKSQUARE</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -4024,7 +6318,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SK_RAPID</t>
+          <t>SK_BLACKSQUARE</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -4034,7 +6328,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>M_SPEEDER</t>
+          <t>M_HIDER</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -4047,7 +6341,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>M_SPEEDER</t>
+          <t>M_HIDER</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -4057,122 +6351,122 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>M_SPEEDER</t>
+          <t>M_HIDER</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>skill</t>
+          <t>monster</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>SK_DASH</t>
+          <t>M_HIDER</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>M_OUMUAMUA</t>
+          <t>M_HIDER</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>recipe</t>
+          <t>monster</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>R_SK_BARRAGE</t>
+          <t>M_HIDER</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>M_OUMUAMUA</t>
+          <t>M_HIDER</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>recipe</t>
+          <t>skill</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>R_SK_BARRAGE</t>
+          <t>SK_HIDE</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>M_OUMUAMUA</t>
+          <t>M_BLACKTRIANGLE</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>recipe</t>
+          <t>monster</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>R_SK_OUMUAMUA</t>
+          <t>M_BLACKTRIANGLE</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>M_OUMUAMUA</t>
+          <t>M_BLACKTRIANGLE</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>recipe</t>
+          <t>monster</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>R_SK_BARRAGE</t>
+          <t>M_BLACKTRIANGLE</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>M_OUMUAMUA</t>
+          <t>M_BLACKTRIANGLE</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -4180,12 +6474,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>recipe</t>
+          <t>monster</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>R_SK_OUMUAMUA</t>
+          <t>M_BLACKTRIANGLE</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -4195,28 +6489,419 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>M_BLACKTRIANGLE</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>skill</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>SK_RAPID</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>M_SPEEDER</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>monster</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>M_SPEEDER</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>M_SPEEDER</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>monster</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>M_SPEEDER</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>M_SPEEDER</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>skill</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>SK_DASH</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>M_OUMUAMUA</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>3</v>
-      </c>
-      <c r="C16" t="inlineStr">
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="inlineStr">
         <is>
           <t>recipe</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>R_SK_BARRAGE</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>M_OUMUAMUA</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>recipe</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>R_SK_BARRAGE</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>M_OUMUAMUA</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>recipe</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>R_SK_OUMUAMUA</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>M_OUMUAMUA</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>recipe</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>R_SK_BARRAGE</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>M_OUMUAMUA</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>recipe</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>R_SK_OUMUAMUA</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>M_OUMUAMUA</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>recipe</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
         <is>
           <t>R_M_OUMUAMUA</t>
         </is>
       </c>
-      <c r="E16" t="n">
+      <c r="E25" t="n">
         <v>0.2</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>M_HAMMER</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>monster</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>M_HAMMER</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>M_HAMMER</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>monster</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>M_HAMMER</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>M_HAMMER</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>monster</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>M_HAMMER</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>M_HAMMER</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>skill</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>SK_HEAVY_STRIKE</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>monster</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>monster</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>monster</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>M_POZ</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>3</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>skill</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>SK_POISON_SECRETION</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E16"/>
+  <autoFilter ref="A1:E33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Add character sprites and markdown database
</commit_message>
<xml_diff>
--- a/NULL_game_db.xlsx
+++ b/NULL_game_db.xlsx
@@ -4632,7 +4632,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>STAGE_002</t>
+          <t>STAGE_001</t>
         </is>
       </c>
     </row>
@@ -4696,7 +4696,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>STAGE_002</t>
+          <t>STAGE_001</t>
         </is>
       </c>
     </row>
@@ -4787,10 +4787,14 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>always</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>clear</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>STAGE_004</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4847,10 +4851,14 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>always</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+          <t>clear</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>STAGE_006</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">

</xml_diff>